<commit_message>
Update disaster map Excel data
</commit_message>
<xml_diff>
--- a/data/disaster_map_data.xlsx
+++ b/data/disaster_map_data.xlsx
@@ -2795,11 +2795,11 @@
         <v>5732</v>
       </c>
       <c r="H14" s="29">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="I14" s="30">
         <f>SUM(B14:H14)</f>
-        <v>19717</v>
+        <v>19617</v>
       </c>
     </row>
     <row r="15" spans="1:9">

</xml_diff>